<commit_message>
- Added dayNotes field to MealPlan model for storing notes keyed by date. - Added meal plan naming - Enhanced GroceryPage component with loading state and improved UI for displaying grocery lists. - Improved API routes for meal plans and grocery lists, including new PATCH endpoints for updating grocery items and plan metadata.
</commit_message>
<xml_diff>
--- a/Plans/MP-backlog-epics-3-28-26.xlsx
+++ b/Plans/MP-backlog-epics-3-28-26.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jresetco/Documents/jrcode/meal-planner/Plans/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB99BC74-024D-2043-9C2C-84D63F7930D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{0451432B-DE77-9F41-885C-927DBA417224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3260" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{FACB6627-D9F0-1142-BBD7-CA4FCE3CCED8}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19740" xr2:uid="{FACB6627-D9F0-1142-BBD7-CA4FCE3CCED8}"/>
   </bookViews>
   <sheets>
     <sheet name="backlog-epics" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'backlog-epics'!$A$1:$H$49</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="145">
   <si>
     <t>Epic</t>
   </si>
@@ -55,9 +58,6 @@
     <t>Replace confirm() with Dialog + textarea for guidance text fed to AI</t>
   </si>
   <si>
-    <t>High</t>
-  </si>
-  <si>
     <t>Small</t>
   </si>
   <si>
@@ -133,9 +133,6 @@
     <t>Add meal components link to navigation</t>
   </si>
   <si>
-    <t>Low</t>
-  </si>
-  <si>
     <t>Grocery List QoL</t>
   </si>
   <si>
@@ -283,18 +280,12 @@
     <t>Mobile-friendly layouts for all pages</t>
   </si>
   <si>
-    <t>‚Äî</t>
-  </si>
-  <si>
     <t>Large</t>
   </si>
   <si>
     <t>P2 / ENH B8</t>
   </si>
   <si>
-    <t>Parked</t>
-  </si>
-  <si>
     <t>Progressive Web App</t>
   </si>
   <si>
@@ -331,9 +322,6 @@
     <t>Nutritional info tracking per meal</t>
   </si>
   <si>
-    <t>Cut</t>
-  </si>
-  <si>
     <t>Daily/weekly nutritional summaries</t>
   </si>
   <si>
@@ -392,13 +380,91 @@
   </si>
   <si>
     <t>P1.0-I.1</t>
+  </si>
+  <si>
+    <t>DONE - Remove</t>
+  </si>
+  <si>
+    <t>CUT - Remove</t>
+  </si>
+  <si>
+    <t>1 - Very High</t>
+  </si>
+  <si>
+    <t>2- High</t>
+  </si>
+  <si>
+    <t>4 - Medium</t>
+  </si>
+  <si>
+    <t>5 - Medium-Low</t>
+  </si>
+  <si>
+    <t>6 - Low</t>
+  </si>
+  <si>
+    <t>Bug - grocery list contains removed meals in item subtext</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root cause is clear: GET /api/plans/[id]/grocery returns a cached GroceryList when one exists, and no meal-plan mutation deletes that list—so mealNames can reference recipes from an older plan (e.g. after swapping off “Instant Pot Spring Risotto”). A secondary issue: the AI can mis-attribute mealNames because they’re free-form strings with no validation against the meal set. Example of issue here: Some grocery list items reference recipes that are not in the actual meal plan, it kept pulling in instant pot spring risotto, even though this was not in the list: http://localhost:3000/plans/cmnb9wods001aku062yrr1ajz </t>
+  </si>
+  <si>
+    <t>Add visible page for excluded items next to grocery list</t>
+  </si>
+  <si>
+    <t>ON grocery list page, show a tab on the right-hand side that shows all of the items that are hidden (e.g. items found in always available pantry)</t>
+  </si>
+  <si>
+    <t>Enhance pantry</t>
+  </si>
+  <si>
+    <t>Add Pantry tab</t>
+  </si>
+  <si>
+    <t>3 - Medium High</t>
+  </si>
+  <si>
+    <t>Add the ability to set a more general groupings of items that will be considered as already available in the grocery list (e.g. "oil" can be used to hide any type of oil) or hide all spices, for example</t>
+  </si>
+  <si>
+    <t>Add auto-substitutions section</t>
+  </si>
+  <si>
+    <t>Add a page that allows me to set automatic substitutions (e.g. every time it says 1 cup white wine; substitue 1 cup apple juice, etc)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enhanced Pantry Staples </t>
+  </si>
+  <si>
+    <t>Add a new navigation page (available on left-hand side) for "Pantry" that currently only displays the "Pantry Staples" functionality.</t>
+  </si>
+  <si>
+    <t>Add merged ingredients management</t>
+  </si>
+  <si>
+    <t>Make Meal planning GenAI Prompt visible and editable in the Settings page</t>
+  </si>
+  <si>
+    <t>Allow me to see and modify the prompt that is being used to generate meals, ensuring proper guardrails so that I do not accidentally remove ingredients/rules/etc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create simple implementation to allow me to better define some basic rules for easier merging/combining of ingredients.  For example, if I wanted to always have soy sauce, dark soy sauce, light soy sauce, low sodium soy sauce, etc all just merge down into soy sauce, without spelling that out for the engine.  Tell me - 1, how this merging works today and come up with a simple implementation plan for this. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enhanced ingredient quantity merging </t>
+  </si>
+  <si>
+    <t>Add logic around how to merge/handle varying measurement types (e.g. cups vs ounces vs counts)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -529,6 +595,19 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -875,8 +954,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1232,11 +1312,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D47915BA-D129-1A46-888E-1D097FF519AE}">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="33.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="98.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.5" customWidth="1"/>
+    <col min="2" max="2" width="5.83203125" customWidth="1"/>
+    <col min="3" max="3" width="31" customWidth="1"/>
+    <col min="4" max="4" width="78.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -1267,1045 +1349,1187 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>126</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="E2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>127</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F3" t="s">
         <v>11</v>
       </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>121</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>121</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="H5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>129</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>130</v>
       </c>
       <c r="E6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" t="s">
-        <v>24</v>
+        <v>133</v>
       </c>
       <c r="H6" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>139</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>142</v>
       </c>
       <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" t="s">
-        <v>24</v>
+        <v>123</v>
       </c>
       <c r="H7" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>143</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>144</v>
       </c>
       <c r="E8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" t="s">
-        <v>24</v>
+        <v>123</v>
       </c>
       <c r="H8" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>131</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>132</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>138</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" t="s">
-        <v>24</v>
+        <v>122</v>
       </c>
       <c r="H9" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>131</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>137</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" t="s">
-        <v>24</v>
-      </c>
-      <c r="H10" t="s">
-        <v>14</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11">
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>37</v>
+        <v>122</v>
       </c>
       <c r="F11" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="E12" t="s">
+        <v>122</v>
+      </c>
+      <c r="F12" t="s">
         <v>11</v>
       </c>
-      <c r="F12" t="s">
-        <v>12</v>
-      </c>
       <c r="G12" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="H12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="E13" t="s">
-        <v>11</v>
+        <v>122</v>
       </c>
       <c r="F13" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G13" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="H13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>122</v>
       </c>
       <c r="F14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G14" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="H14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="B15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="E15" t="s">
-        <v>20</v>
+        <v>122</v>
       </c>
       <c r="F15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G15" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="H15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>122</v>
       </c>
       <c r="F16" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G16" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="H16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="E17" t="s">
-        <v>20</v>
+        <v>122</v>
       </c>
       <c r="F17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G17" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="H17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>8</v>
       </c>
       <c r="B18">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="D18" t="s">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E18" t="s">
+        <v>123</v>
+      </c>
+      <c r="F18" t="s">
         <v>11</v>
       </c>
-      <c r="F18" t="s">
-        <v>20</v>
-      </c>
       <c r="G18" t="s">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="H18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>8</v>
       </c>
       <c r="B19">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>140</v>
       </c>
       <c r="D19" t="s">
-        <v>63</v>
+        <v>141</v>
       </c>
       <c r="E19" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="F19" t="s">
-        <v>12</v>
-      </c>
-      <c r="G19" t="s">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="H19" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B20">
         <v>5</v>
       </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E20" t="s">
-        <v>37</v>
+        <v>123</v>
       </c>
       <c r="F20" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G20" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E21" t="s">
+        <v>123</v>
+      </c>
+      <c r="F21" t="s">
         <v>11</v>
       </c>
-      <c r="F21" t="s">
-        <v>20</v>
-      </c>
       <c r="G21" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="H21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B22">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C22" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="D22" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="E22" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="F22" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="G22" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="H22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B23">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C23" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="E23" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="F23" t="s">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="G23" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="H23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B24">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C24" t="s">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="D24" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="E24" t="s">
-        <v>37</v>
+        <v>124</v>
       </c>
       <c r="F24" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="G24" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="H24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B25">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C25" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="D25" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="E25" t="s">
-        <v>20</v>
+        <v>124</v>
       </c>
       <c r="F25" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="G25" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="H25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B26">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C26" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="D26" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="E26" t="s">
-        <v>20</v>
+        <v>124</v>
       </c>
       <c r="F26" t="s">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="G26" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B27">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>85</v>
+        <v>135</v>
       </c>
       <c r="D27" t="s">
-        <v>86</v>
+        <v>136</v>
       </c>
       <c r="E27" t="s">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="F27" t="s">
-        <v>88</v>
-      </c>
-      <c r="G27" t="s">
-        <v>89</v>
-      </c>
-      <c r="H27" t="s">
-        <v>90</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="B28">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="D28" t="s">
-        <v>92</v>
+        <v>48</v>
       </c>
       <c r="E28" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F28" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="G28" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="H28" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="B29">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="D29" t="s">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="E29" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F29" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G29" t="s">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="H29" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="B30">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>97</v>
+        <v>53</v>
       </c>
       <c r="D30" t="s">
-        <v>98</v>
+        <v>54</v>
       </c>
       <c r="E30" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F30" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="G30" t="s">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="H30" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="B31">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>99</v>
+        <v>63</v>
       </c>
       <c r="D31" t="s">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="E31" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F31" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="G31" t="s">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="H31" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B32">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C32" t="s">
-        <v>101</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
       <c r="E32" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F32" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="G32" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="H32" t="s">
-        <v>103</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B33">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C33" t="s">
-        <v>104</v>
+        <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="E33" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F33" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="G33" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="H33" t="s">
-        <v>103</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B34">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C34" t="s">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="D34" t="s">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="E34" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G34" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="H34" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B35">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C35" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="D35" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="E35" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F35" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G35" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="H35" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B36">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C36" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
       <c r="D36" t="s">
-        <v>111</v>
+        <v>77</v>
       </c>
       <c r="E36" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F36" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="G36" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="H36" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B37">
         <v>8</v>
       </c>
       <c r="C37" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="D37" t="s">
-        <v>113</v>
+        <v>88</v>
       </c>
       <c r="E37" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F37" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="G37" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H37" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B38">
         <v>8</v>
       </c>
       <c r="C38" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="D38" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="E38" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F38" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H38" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B39">
         <v>8</v>
       </c>
       <c r="C39" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="D39" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="E39" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F39" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="G39" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H39" t="s">
-        <v>90</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B40">
         <v>8</v>
       </c>
       <c r="C40" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="D40" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="E40" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G40" t="s">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="H40" t="s">
-        <v>103</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B41">
         <v>8</v>
       </c>
       <c r="C41" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="D41" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="E41" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="F41" t="s">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="G41" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="H41" t="s">
-        <v>103</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>109</v>
+      </c>
+      <c r="D42" t="s">
+        <v>110</v>
+      </c>
+      <c r="E42" t="s">
+        <v>125</v>
+      </c>
+      <c r="F42" t="s">
+        <v>19</v>
+      </c>
+      <c r="G42" t="s">
+        <v>89</v>
+      </c>
+      <c r="H42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>82</v>
+      </c>
+      <c r="B43">
+        <v>8</v>
+      </c>
+      <c r="C43" t="s">
+        <v>111</v>
+      </c>
+      <c r="D43" t="s">
+        <v>112</v>
+      </c>
+      <c r="E43" t="s">
+        <v>125</v>
+      </c>
+      <c r="F43" t="s">
+        <v>85</v>
+      </c>
+      <c r="G43" t="s">
+        <v>89</v>
+      </c>
+      <c r="H43" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>8</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" t="s">
+        <v>15</v>
+      </c>
+      <c r="F44" t="s">
+        <v>11</v>
+      </c>
+      <c r="G44" t="s">
+        <v>16</v>
+      </c>
+      <c r="H44" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>8</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" t="s">
+        <v>18</v>
+      </c>
+      <c r="F45" t="s">
+        <v>11</v>
+      </c>
+      <c r="G45" t="s">
+        <v>16</v>
+      </c>
+      <c r="H45" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>78</v>
+      </c>
+      <c r="B46">
+        <v>7</v>
+      </c>
+      <c r="C46" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46" t="s">
+        <v>80</v>
+      </c>
+      <c r="G46" t="s">
+        <v>81</v>
+      </c>
+      <c r="H46" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>82</v>
+      </c>
+      <c r="B47">
+        <v>8</v>
+      </c>
+      <c r="C47" t="s">
+        <v>107</v>
+      </c>
+      <c r="D47" t="s">
+        <v>108</v>
+      </c>
+      <c r="F47" t="s">
+        <v>11</v>
+      </c>
+      <c r="G47" t="s">
+        <v>89</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>82</v>
+      </c>
+      <c r="B48">
+        <v>8</v>
+      </c>
+      <c r="C48" t="s">
+        <v>113</v>
+      </c>
+      <c r="D48" t="s">
+        <v>114</v>
+      </c>
+      <c r="G48" t="s">
+        <v>115</v>
+      </c>
+      <c r="H48" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>82</v>
+      </c>
+      <c r="B49">
+        <v>8</v>
+      </c>
+      <c r="C49" t="s">
+        <v>116</v>
+      </c>
+      <c r="D49" t="s">
+        <v>117</v>
+      </c>
+      <c r="G49" t="s">
+        <v>118</v>
+      </c>
+      <c r="H49" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H49" xr:uid="{D47915BA-D129-1A46-888E-1D097FF519AE}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H49">
+      <sortCondition ref="E1:E49"/>
+    </sortState>
+  </autoFilter>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>